<commit_message>
Fix date formatting to DD-MMM-YY in output and test file
Dates in output Excel now display as 03-Mar-20 instead of
2020-03-03 00:00:00. Test FRA file updated to match reference
data exactly (5 rows, RT=12).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_input_fra.xlsx
+++ b/test_input_fra.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="DD-MMM-YY"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,7 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AZ11"/>
+  <dimension ref="B1:AZ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,31 +489,31 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AC2" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="AD2" t="n">
         <v>1</v>
       </c>
       <c r="AE2" s="1" t="n">
-        <v>36692</v>
+        <v>42066</v>
       </c>
       <c r="AF2" s="1" t="n">
-        <v>45823</v>
+        <v>43893</v>
       </c>
       <c r="AH2" s="1" t="n">
-        <v>45823</v>
+        <v>43893</v>
       </c>
       <c r="AS2" t="n">
-        <v>500000</v>
+        <v>462500</v>
       </c>
       <c r="AW2" s="1" t="n">
-        <v>45458</v>
+        <v>46084</v>
       </c>
       <c r="AZ2" t="n">
-        <v>47050</v>
+        <v>92500</v>
       </c>
     </row>
     <row r="3">
@@ -527,31 +528,31 @@
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="AC3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AD3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE3" s="1" t="n">
-        <v>38421</v>
+        <v>42066</v>
       </c>
       <c r="AF3" s="1" t="n">
-        <v>45726</v>
+        <v>45719</v>
       </c>
       <c r="AH3" s="1" t="n">
-        <v>45726</v>
+        <v>45719</v>
       </c>
       <c r="AS3" t="n">
-        <v>300000</v>
+        <v>291010</v>
       </c>
       <c r="AW3" s="1" t="n">
-        <v>45361</v>
+        <v>46084</v>
       </c>
       <c r="AZ3" t="n">
-        <v>8952</v>
+        <v>29101</v>
       </c>
     </row>
     <row r="4">
@@ -566,31 +567,31 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AC4" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="AD4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE4" s="1" t="n">
-        <v>40179</v>
+        <v>42077</v>
       </c>
       <c r="AF4" s="1" t="n">
-        <v>45658</v>
+        <v>43904</v>
       </c>
       <c r="AH4" s="1" t="n">
-        <v>45658</v>
+        <v>43904</v>
       </c>
       <c r="AS4" t="n">
-        <v>200000</v>
+        <v>160183</v>
       </c>
       <c r="AW4" s="1" t="n">
-        <v>45292</v>
+        <v>46095</v>
       </c>
       <c r="AZ4" t="n">
-        <v>1310</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="5">
@@ -605,31 +606,31 @@
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="AC5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AD5" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AE5" s="1" t="n">
-        <v>38534</v>
+        <v>42063</v>
       </c>
       <c r="AF5" s="1" t="n">
-        <v>44013</v>
+        <v>45716</v>
       </c>
       <c r="AH5" s="1" t="n">
-        <v>45839</v>
+        <v>45716</v>
       </c>
       <c r="AS5" t="n">
-        <v>400000</v>
+        <v>291010</v>
       </c>
       <c r="AW5" s="1" t="n">
-        <v>45474</v>
+        <v>46081</v>
       </c>
       <c r="AZ5" t="n">
-        <v>30000</v>
+        <v>29101</v>
       </c>
     </row>
     <row r="6">
@@ -644,226 +645,31 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AC6" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="AD6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE6" s="1" t="n">
-        <v>36770</v>
+        <v>42066</v>
       </c>
       <c r="AF6" s="1" t="n">
-        <v>43344</v>
+        <v>43893</v>
       </c>
       <c r="AH6" s="1" t="n">
-        <v>45901</v>
+        <v>44623</v>
       </c>
       <c r="AS6" t="n">
-        <v>250000</v>
+        <v>176547</v>
       </c>
       <c r="AW6" s="1" t="n">
-        <v>45536</v>
+        <v>46084</v>
       </c>
       <c r="AZ6" t="n">
-        <v>2213</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>IF</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>MSB</t>
-        </is>
-      </c>
-      <c r="AB7" t="n">
-        <v>30</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>30</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE7" s="1" t="n">
-        <v>34790</v>
-      </c>
-      <c r="AF7" s="1" t="n">
-        <v>45748</v>
-      </c>
-      <c r="AH7" s="1" t="n">
-        <v>45748</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>600000</v>
-      </c>
-      <c r="AW7" s="1" t="n">
-        <v>45383</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SU</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>FSP</t>
-        </is>
-      </c>
-      <c r="AB8" t="n">
-        <v>15</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>15</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE8" s="1" t="n">
-        <v>40483</v>
-      </c>
-      <c r="AF8" s="1" t="n">
-        <v>44866</v>
-      </c>
-      <c r="AH8" s="1" t="n">
-        <v>45962</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>150000</v>
-      </c>
-      <c r="AW8" s="1" t="n">
-        <v>45597</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>IF</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>FSP</t>
-        </is>
-      </c>
-      <c r="AB9" t="n">
-        <v>30</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>30</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>12</v>
-      </c>
-      <c r="AE9" s="1" t="n">
-        <v>34745</v>
-      </c>
-      <c r="AF9" s="1" t="n">
-        <v>45703</v>
-      </c>
-      <c r="AH9" s="1" t="n">
-        <v>45703</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>800000</v>
-      </c>
-      <c r="AW9" s="1" t="n">
-        <v>45337</v>
-      </c>
-      <c r="AZ9" t="n">
-        <v>5500</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>FSP</t>
-        </is>
-      </c>
-      <c r="AB10" t="n">
-        <v>20</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>20</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE10" s="1" t="n">
-        <v>38584</v>
-      </c>
-      <c r="AF10" s="1" t="n">
-        <v>45158</v>
-      </c>
-      <c r="AH10" s="1" t="n">
-        <v>45889</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>350000</v>
-      </c>
-      <c r="AW10" s="1" t="n">
-        <v>45524</v>
-      </c>
-      <c r="AZ10" t="n">
-        <v>6500</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IF</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>FSP</t>
-        </is>
-      </c>
-      <c r="AB11" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE11" s="1" t="n">
-        <v>42125</v>
-      </c>
-      <c r="AF11" s="1" t="n">
-        <v>45778</v>
-      </c>
-      <c r="AH11" s="1" t="n">
-        <v>45778</v>
-      </c>
-      <c r="AS11" t="n">
-        <v>100000</v>
-      </c>
-      <c r="AW11" s="1" t="n">
-        <v>45413</v>
-      </c>
-      <c r="AZ11" t="n">
-        <v>8000</v>
+        <v>25221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>